<commit_message>
Blank template: defaults filled in, Badgaon examples beside the blanks
Check dam: evaporation 5 mm/day, weir coefficient 1.6 and exponent 1.5 are
filled in (the calculator's own defaults). The dam's levels, the pond
survey and the readings stay blank, since a default there would silently
give a wrong answer; each sheet shows the Badgaon values in example columns
to the right instead. The importer reads the first matching column, and now
counts a row as skipped only if it has something in a column it reads, so
the examples are never imported and raise no warning. Tests: the blank
template's defaults, and a filled-in one importing only the user's values.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/checkdamcal-template.xlsx
+++ b/examples/checkdamcal-template.xlsx
@@ -68,8 +68,9 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="60" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -401,7 +402,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C9"/>
+  <dimension ref="A1:C11"/>
   <cols>
     <col min="1" max="1" width="16.83203125" customWidth="1"/>
     <col min="2" max="2" width="110.83203125" customWidth="1"/>
@@ -423,65 +424,76 @@
         <v>Keep the sheet names and the header rows as they are. Leave a cell blank if you don’t have the value.</v>
       </c>
     </row>
+    <row r="5">
+      <c r="A5" t="str">
+        <v>Evaporation and the two weir values are filled in with the usual defaults: change them if you have your own.</v>
+      </c>
+    </row>
     <row r="6">
       <c r="A6" t="str">
-        <v>Sheet</v>
-      </c>
-      <c r="B6" t="str">
-        <v>What goes in it</v>
-      </c>
-      <c r="C6" t="str">
-        <v>How often</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" t="str">
-        <v>Check dam</v>
-      </c>
-      <c r="B7" t="str">
-        <v>The heights of the gauge board’s 0 cm mark and of the spillway, and the spillway’s length (all in metres, from the same reference point). Evaporation in mm per day. Catchment area in hectares (optional).</v>
-      </c>
-      <c r="C7" t="str">
-        <v>Once</v>
+        <v>The “Example (Badgaon 2014)” columns on the right show what goes where, from the Badgaon check dam. They are never imported: type your own values in the columns on the left.</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
-        <v>Pond survey</v>
+        <v>Sheet</v>
       </c>
       <c r="B8" t="str">
-        <v>The water-surface area at several levels, from the lowest point of the pond (area 0) up to a little above the spillway. Volume is optional: leave it blank to have it worked out.</v>
+        <v>What goes in it</v>
       </c>
       <c r="C8" t="str">
-        <v>Once</v>
+        <v>How often</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="str">
+        <v>Check dam</v>
+      </c>
+      <c r="B9" t="str">
+        <v>The heights of the gauge board’s 0 cm mark and of the spillway, and the spillway’s length (all in metres, from the same reference point). Evaporation in mm per day. Catchment area in hectares (optional).</v>
+      </c>
+      <c r="C9" t="str">
+        <v>Once</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="str">
+        <v>Pond survey</v>
+      </c>
+      <c r="B10" t="str">
+        <v>The water-surface area at several levels, from the lowest point of the pond (area 0) up to a little above the spillway. Volume is optional: leave it blank to have it worked out.</v>
+      </c>
+      <c r="C10" t="str">
+        <v>Once</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="str">
         <v>Daily readings</v>
       </c>
-      <c r="B9" t="str">
+      <c r="B11" t="str">
         <v>One row per day: the date, the gauge-board reading in cm, and the rainfall in mm (blank on dry days). Level override is optional: type a level in metres only to correct a reading.</v>
       </c>
-      <c r="C9" t="str">
+      <c r="C11" t="str">
         <v>Every day</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C9"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:C11"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D8"/>
+  <dimension ref="A1:E8"/>
   <cols>
     <col min="1" max="1" width="20.83203125" customWidth="1"/>
     <col min="2" max="2" width="10.83203125" customWidth="1"/>
     <col min="3" max="3" width="8.83203125" customWidth="1"/>
     <col min="4" max="4" width="70.83203125" customWidth="1"/>
+    <col min="5" max="5" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -497,6 +509,9 @@
       <c r="D1" t="str">
         <v>Notes</v>
       </c>
+      <c r="E1" t="str">
+        <v>Example (Badgaon 2014)</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="str">
@@ -508,6 +523,9 @@
       <c r="D2" t="str">
         <v>Height of the gauge board’s 0 cm mark</v>
       </c>
+      <c r="E2">
+        <v>98.43</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="str">
@@ -519,6 +537,9 @@
       <c r="D3" t="str">
         <v>Height of the top of the overflow section (water spills above it)</v>
       </c>
+      <c r="E3">
+        <v>100</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="str">
@@ -530,16 +551,25 @@
       <c r="D4" t="str">
         <v>Width of the overflow section, across the stream</v>
       </c>
+      <c r="E4">
+        <v>12.7</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="str">
         <v>Evaporation</v>
       </c>
+      <c r="B5">
+        <v>5</v>
+      </c>
       <c r="C5" t="str">
         <v>mm/day</v>
       </c>
       <c r="D5" t="str">
         <v>Water lost to the air from the pond each day</v>
+      </c>
+      <c r="E5">
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -552,43 +582,62 @@
       <c r="D6" t="str">
         <v>Optional: land that drains into the check dam</v>
       </c>
+      <c r="E6">
+        <v>338.31</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="str">
         <v>Weir coefficient</v>
       </c>
+      <c r="B7">
+        <v>1.6</v>
+      </c>
       <c r="C7" t="str">
         <v/>
       </c>
       <c r="D7" t="str">
         <v>Advanced: C₁ in Q = C₁·L₁·H^a₁ (m³/s); the workbook uses 1.6</v>
+      </c>
+      <c r="E7">
+        <v>1.6</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="str">
         <v>Weir exponent</v>
       </c>
+      <c r="B8">
+        <v>1.5</v>
+      </c>
       <c r="C8" t="str">
         <v/>
       </c>
       <c r="D8" t="str">
         <v>Advanced: a₁; 1.5 for a broad-crested weir</v>
       </c>
+      <c r="E8">
+        <v>1.5</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:E8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:C1"/>
+  <dimension ref="A1:G8"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
+    <col min="4" max="4" width="3.83203125" customWidth="1"/>
+    <col min="5" max="5" width="30.83203125" customWidth="1"/>
+    <col min="6" max="6" width="18.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -601,22 +650,115 @@
       <c r="C1" t="str">
         <v>Volume (m³)</v>
       </c>
+      <c r="D1" t="str">
+        <v/>
+      </c>
+      <c r="E1" t="str">
+        <v>Example (Badgaon 2014): level (m)</v>
+      </c>
+      <c r="F1" t="str">
+        <v>Example: area (m²)</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Example: volume (m³)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="E2">
+        <v>97.7</v>
+      </c>
+      <c r="F2">
+        <v>0</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="E3">
+        <v>98</v>
+      </c>
+      <c r="F3">
+        <v>2247</v>
+      </c>
+      <c r="G3">
+        <v>225</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="E4">
+        <v>98.5</v>
+      </c>
+      <c r="F4">
+        <v>10723.5</v>
+      </c>
+      <c r="G4">
+        <v>3467.625</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="E5">
+        <v>99</v>
+      </c>
+      <c r="F5">
+        <v>19200</v>
+      </c>
+      <c r="G5">
+        <v>10948.5</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="E6">
+        <v>99.5</v>
+      </c>
+      <c r="F6">
+        <v>27676.5</v>
+      </c>
+      <c r="G6">
+        <v>22667.625</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="E7">
+        <v>100</v>
+      </c>
+      <c r="F7">
+        <v>39000</v>
+      </c>
+      <c r="G7">
+        <v>39336.75</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="E8">
+        <v>100.5</v>
+      </c>
+      <c r="F8">
+        <v>44629.5</v>
+      </c>
+      <c r="G8">
+        <v>60244.125</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:C1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:G8"/>
   </ignoredErrors>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:D1"/>
+  <dimension ref="A1:H11"/>
   <cols>
     <col min="1" max="1" width="12.83203125" customWidth="1"/>
     <col min="2" max="2" width="18.83203125" customWidth="1"/>
     <col min="3" max="3" width="14.83203125" customWidth="1"/>
     <col min="4" max="4" width="18.83203125" customWidth="1"/>
+    <col min="5" max="5" width="3.83203125" customWidth="1"/>
+    <col min="6" max="6" width="28.83203125" customWidth="1"/>
+    <col min="7" max="7" width="20.83203125" customWidth="1"/>
+    <col min="8" max="8" width="22.83203125" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -632,10 +774,120 @@
       <c r="D1" t="str">
         <v>Level override (m)</v>
       </c>
+      <c r="E1" t="str">
+        <v/>
+      </c>
+      <c r="F1" t="str">
+        <v>Example (Badgaon 2014): date</v>
+      </c>
+      <c r="G1" t="str">
+        <v>Example: gauge (cm)</v>
+      </c>
+      <c r="H1" t="str">
+        <v>Example: rainfall (mm)</v>
+      </c>
+    </row>
+    <row r="2">
+      <c r="F2" s="1">
+        <v>41836</v>
+      </c>
+      <c r="G2">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>2.7</v>
+      </c>
+    </row>
+    <row r="3">
+      <c r="F3" s="1">
+        <v>41837</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="F4" s="1">
+        <v>41838</v>
+      </c>
+      <c r="G4">
+        <v>140</v>
+      </c>
+      <c r="H4">
+        <v>9.6</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="F5" s="1">
+        <v>41839</v>
+      </c>
+      <c r="G5">
+        <v>130</v>
+      </c>
+      <c r="H5">
+        <v>34.3</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="F6" s="1">
+        <v>41840</v>
+      </c>
+      <c r="G6">
+        <v>125</v>
+      </c>
+      <c r="H6">
+        <v>58.2</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="F7" s="1">
+        <v>41841</v>
+      </c>
+      <c r="G7">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="F8" s="1">
+        <v>41842</v>
+      </c>
+      <c r="G8">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="F9" s="1">
+        <v>41843</v>
+      </c>
+      <c r="G9">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="F10" s="1">
+        <v>41844</v>
+      </c>
+      <c r="G10">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="F11" s="1">
+        <v>41845</v>
+      </c>
+      <c r="G11">
+        <v>160</v>
+      </c>
+      <c r="H11">
+        <v>26.1</v>
+      </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:D1"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:H11"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>